<commit_message>
fix: make manifest ground truth row-level and exact
</commit_message>
<xml_diff>
--- a/samples/change_orders_sample.xlsx
+++ b/samples/change_orders_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,17 +483,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Daniel Farmer MD</t>
+          <t>Melanie Rogers</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-01-26 06:40:14.381550</t>
+          <t>2026-01-29 14:04:50.381550</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-02-01 06:40:14.381550</t>
+          <t>2026-02-04 14:04:50.381550</t>
         </is>
       </c>
     </row>
@@ -505,37 +505,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Water allow attention floor stay successful career.
-Month whose various behavior window.
-Growth likely store least recent people item.
-Media sing every blood great attorney.</t>
+Month whose various behavior window.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Justin Baldwin</t>
+          <t>Alexandra Humphrey</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2024-07-31 08:50:54.756929</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2024-10-20 08:50:54.756929</t>
-        </is>
-      </c>
+          <t>2024-08-03 16:15:30.756929</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -545,7 +539,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,22 +549,26 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Himself ground simply stop.
-Easy particular Republican quality ask exist break nice.
-Morning product point strategy result country.</t>
+          <t>Letter avoid see name body difficult media.
+Check organization theory participant leave.
+Contain feeling significant data boy easy.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lynn Gomez</t>
+          <t>Samantha Ramirez</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2023-11-11 09:09:57.349159</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>2024-06-10 16:45:48.891043</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2024-07-23 16:45:48.891043</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -580,7 +578,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -590,23 +588,27 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Occur pull thought test.
-Off vote age power along simple.
-Voice away key concern set my.
-Road likely relate chance himself.</t>
+          <t>Series speech hard consumer.
+Seem notice old commercial my assume beyond.
+Company a respond control feeling off.
+Military rock culture.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Melissa Osborne</t>
+          <t>Roy Velazquez</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2024-02-05 02:37:03.153946</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>2024-12-19 17:42:01.186899</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-04-05 17:42:01.186899</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -626,102 +628,100 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Hot practice career high.
+Road likely relate chance himself.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Andrew Crawford</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2023-06-20 07:45:09.213215</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2023-09-28 07:45:09.213215</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CO-000006</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>American apply wish help floor prevent.
 Treatment arm easy home fill new drop.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Amy Kelley</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2023-10-07 09:37:38.338488</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2024-01-15 09:37:38.338488</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CO-000006</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>David Boyle</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2023-10-10 17:02:14.338488</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2024-01-30 17:02:14.338488</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CO-000007</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Evening arm yes type majority article.
 Family join woman truth summer avoid.
 Out deal head far push adult need pick.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Melissa Osborne</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-02-10 16:17:08.432679</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-06-02 16:17:08.432679</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CO-000007</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>rejected</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Serve build happen prevent important.
-Degree game choice many.
-Hope church us contain discussion.
-Former group security outside purpose.</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Amy Kelley</t>
+          <t>Andrew Vasquez</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2024-02-08 07:13:20.248633</t>
+          <t>2026-02-13 23:41:44.432679</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2024-03-11 07:13:20.248633</t>
+          <t>2026-03-17 23:41:44.432679</t>
         </is>
       </c>
     </row>
@@ -743,18 +743,18 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>National option perhaps indeed small international wish.
-Conference remain somebody very it by.</t>
+          <t>Serve build happen prevent important.
+Degree game choice many.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Amy Kelley</t>
+          <t>Wesley Montgomery</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2022-11-08 05:18:25.642472</t>
+          <t>2024-02-11 14:37:56.248633</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -777,25 +777,26 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Focus out property.
-Peace blood million candidate off.
-Happy executive involve win those.
-Former industry game deal work.</t>
+          <t>Experience budget forget father.
+Former group security outside purpose.
+Make little even drive.
+Loss pressure use morning conference remain.
+Very it by radio.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Daniel Farmer MD</t>
+          <t>Kimberly Elliott</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-03-31 15:14:05.441168</t>
+          <t>2023-07-20 06:22:46.644673</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2025-04-23 15:14:05.441168</t>
+          <t>2023-08-12 06:22:46.644673</t>
         </is>
       </c>
     </row>
@@ -812,22 +813,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rather yeah spend place child.</t>
+          <t>Specific student attorney peace blood million.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Amy Kelley</t>
+          <t>Emma Benitez</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2023-12-01 20:26:48.677465</t>
+          <t>2025-09-05 20:00:43.924713</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -840,35 +841,34 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>open</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Executive news dog choice.
-Church them within she significant.</t>
+          <t>Everything major perform site leg.
+Despite feel fire glass.
+Work glass ability early.
+Place child when because executive news dog.
+Treatment still church them.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sylvia Johnston</t>
+          <t>Xavier Bowers</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-05-08 12:53:54.696684</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-07-31 12:53:54.696684</t>
-        </is>
-      </c>
+          <t>2023-01-18 22:05:38.459168</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -878,32 +878,1449 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Able forget education say.
+Hospital poor how wife foot team the plant.
+Drive instead board war.
+Democratic senior property far.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Jason Hendrix</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-06-09 20:24:16.876507</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-08-18 20:24:16.876507</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CO-000013</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Arrive campaign evening affect.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Katherine Taylor</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2024-01-31 22:21:56.951699</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2024-03-20 22:21:56.951699</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CO-000014</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Could mention view hospital think stop member.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Kevin Summers</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2025-06-10 14:55:59.821091</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2025-09-24 14:55:59.821091</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CO-000015</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Wonder economy always enough bit when fly whether.
+Computer few owner hard.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Daniel Farmer MD</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2024-03-12 08:54:44.907228</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2024-05-15 08:54:44.907228</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CO-000016</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Question guy cell place item growth.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Mary Hall</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2023-04-15 10:14:53.150562</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2023-08-10 10:14:53.150562</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CO-000017</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>He name view clearly reach well provide.
+Form friend responsibility follow.
+Room west charge your television great.
+Necessary light worker increase move total range.
+Easy appear interview part.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Alexandra Humphrey</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-05-05 09:47:27.291142</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CO-000018</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Yourself break fill local operation green small.
+Now since treat nothing.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Jennifer Tanner</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-04-05 18:47:41.002856</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CO-000019</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Notice instead start difficult mission seem summer.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Courtney Miller</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2023-02-02 01:33:04.385047</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2023-02-24 01:33:04.385047</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CO-000020</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ok describe within water.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Zachary Schroeder</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-01-03 11:16:27.360620</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CO-000021</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>in-review</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Little could strong hospital poor how.
-Foot team the plant available view.
-Board war rather democratic.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Lynn Gomez</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2022-12-31 11:12:52.492593</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Whatever nice measure reality how concern issue.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>William Ramos</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2025-08-12 18:39:13.224580</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CO-000022</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Worry research different system member drug.
+Set small yeah material.
+Sing suddenly member five push.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Kevin Walker</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2023-05-03 18:22:31.584309</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2023-07-23 18:22:31.584309</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CO-000023</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Shake campaign when staff computer.
+Line although subject window light feeling PM.
+Conference throughout test blue white senior sing.
+Stay trouble mind wear.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Shannon Watts</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2023-11-30 08:11:41.410826</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2024-01-12 08:11:41.410826</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CO-000024</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Second unit economy art seven.
+Less difficult these wrong score region pass.
+Hard agency statement reveal tough find.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Julie Scott</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-05-18 23:49:11.755691</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-06-18 23:49:11.755691</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CO-000025</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Building open clear pay.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Donald Allen</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-05-15 12:36:01.980494</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-08-25 12:36:01.980494</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CO-000026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Black time kind mean middle deep state.
+Wrong while discuss still.
+Positive because trade drop soldier.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Andrew Crawford</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2022-09-10 09:18:14.680968</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CO-000027</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Pass crime respond risk test deep.
+Situation by because about.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Shaun Carrillo</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2022-11-22 21:23:30.381823</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2022-12-06 21:23:30.381823</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CO-000028</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Interesting see herself employee.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Tiffany Moore</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2025-05-11 18:12:50.003308</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2025-07-30 18:12:50.003308</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CO-000029</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Make hear week in.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Amy Davis</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2023-11-07 02:17:31.526746</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2023-12-21 02:17:31.526746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CO-000030</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Treat edge pretty six best stay.
+Case book federal card.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sheryl Singleton</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2023-12-12 00:01:29.058094</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2023-12-01 00:01:29.058094</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CO-000031</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>in-review</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Future cell suffer practice debate play.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Joyce Mcdonald</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2024-08-06 10:51:45.159406</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CO-000032</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>in-review</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Story debate win arrive.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Emma Benitez</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2024-02-14 15:29:11.180352</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CO-000033</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Security fine probably war employee responsibility defense.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Joseph Anderson</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2022-09-01 07:49:21.123763</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2022-09-26 07:49:21.123763</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CO-000034</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Someone agreement sit his friend blue.
+Commercial less lead election popular should.
+Section food buy along main financial arm range.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Jennifer Johns</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2023-02-12 05:16:25.321009</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2023-03-26 05:16:25.321009</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CO-000035</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Cover energy history candidate.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Kelly Cooper</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2025-07-23 13:42:12.517858</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2025-08-14 13:42:12.517858</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CO-000036</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Until second hair success effort official environmental.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Donald Allen</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2024-11-27 15:39:02.168071</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2025-03-01 15:39:02.168071</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CO-000037</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Dream consider them consider fact hour.
+Finally sometimes court mention.
+Piece they evidence art mouth.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Lindsay Salinas</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2025-06-24 13:09:59.141813</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2025-06-01 13:09:59.141813</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CO-000038</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Technology court say between defense wrong.
+Music quickly do write skin customer actually.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Brian Turner</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2023-06-20 00:05:49.060127</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2023-10-11 00:05:49.060127</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CO-000039</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Research drug analysis certainly keep stage position.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Antonio Hamilton</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2023-02-13 13:47:44.716957</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2023-03-18 13:47:44.716957</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CO-000040</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>in-review</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Care car bill hotel case cup strong.
+Leader friend enough sense change allow.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Kayla Ramos</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2025-01-16 05:41:04.406902</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CO-000041</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Her eight soon single first.
+Other look popular behind air tree anything.
+Year second shake last expect technology sense.
+Prevent energy agent.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Alan Brooks</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2022-11-20 03:51:42.368827</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2022-11-25 03:51:42.368827</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CO-000042</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>in-review</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Meet site his line return.
+Ten thousand would age hot back look.
+Maintain tax member page something seat.
+Population fear stage eight hospital view nor teacher.
+Like population trade candidate big idea direction.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Xavier Bowers</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2025-03-06 08:53:01.912190</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CO-000043</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Prepare improve cold away.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Tiffany Moore</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2023-04-16 12:03:41.227547</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2023-06-25 12:03:41.227547</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CO-000044</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Go without ten job special.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Alan Brooks</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2023-06-19 07:40:21.487398</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2023-09-20 07:40:21.487398</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CO-000045</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Second bag discuss minute enough.
+Board step church campaign.
+Impact glass chance traditional least force.
+Trade expert popular may suffer thousand that people.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Gregory Taylor</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2024-12-06 00:09:21.376047</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2025-01-21 00:09:21.376047</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CO-000046</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>in-review</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Tree various recently act loss west PM size.
+Close model two card.
+Stock black hope past hard.
+Continue TV deep write born outside.
+Which family child although consumer chance.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>David Miller</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:59:06.129110</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CO-000047</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Check behind front government truth service result face.
+Example dinner win seem matter anything husband hit.
+Loss according down media approach.
+Discuss total concern laugh may idea.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Richard Wright III</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2025-04-23 13:49:10.054613</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2025-08-18 13:49:10.054613</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CO-000048</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Score site by stock certainly bring.
+Effect myself because major phone.
+Skill still generation bag.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Shannon Watts</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2023-03-08 11:20:22.945730</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2023-05-05 11:20:22.945730</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CO-000049</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Guess cold skin go PM.
+Few most market public.
+Care wrong manager matter huge magazine.
+Fish father system even with.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Jennifer Carpenter</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2023-05-06 19:54:14.906837</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2023-08-28 19:54:14.906837</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CO-000050</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Reflect situation work difference public capital together.
+Article space seek trouble suffer degree.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Molly Carter</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:43:15.688026</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:43:15.688026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>